<commit_message>
ARD statistics from a catalog, formats and stat_fmt; Studies list one line a study
- company standards sheet ard_statistics: the statistics an analysis may ask
  for (cards' own and computed ones: CV, SE, geometric mean/SD/CV and CIs,
  log-scale mean/SD, percentiles, CI of the mean ...), each with its default
  stat_fmt format; ard_methods gains formats, ttest/wilcox/chisq/fisher
- analyses gain formats (mean=xx.x | p=xx.x% | AGE:sd=xx.xx | pvalue); the
  ARD program formats every result (stat_fmt) and keeps only the statistics
  asked of methods that give a fixed set (mean_ci, proportion_ci, tests)
- ARD tab: statistics and formats picker per analysis, catalog table
- Studies: no folder column (the study root above the list), reports count,
  selected study summarised on the right, double-click opens

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/standards/company_standards_draft.xlsx
+++ b/inst/standards/company_standards_draft.xlsx
@@ -16,20 +16,21 @@
     <sheet name="statistics" sheetId="7" r:id="rId7"/>
     <sheet name="categorical_formats" sheetId="8" r:id="rId8"/>
     <sheet name="ard_methods" sheetId="9" r:id="rId9"/>
-    <sheet name="listing_types" sheetId="10" r:id="rId10"/>
-    <sheet name="populations" sheetId="11" r:id="rId11"/>
-    <sheet name="datasets" sheetId="12" r:id="rId12"/>
-    <sheet name="default_header" sheetId="13" r:id="rId13"/>
-    <sheet name="default_footer" sheetId="14" r:id="rId14"/>
-    <sheet name="default_cells" sheetId="15" r:id="rId15"/>
-    <sheet name="default_layout" sheetId="16" r:id="rId16"/>
-    <sheet name="default_columns" sheetId="17" r:id="rId17"/>
-    <sheet name="default_style" sheetId="18" r:id="rId18"/>
-    <sheet name="default_col_header" sheetId="19" r:id="rId19"/>
-    <sheet name="default_report" sheetId="20" r:id="rId20"/>
-    <sheet name="default_page" sheetId="21" r:id="rId21"/>
-    <sheet name="default_titles" sheetId="22" r:id="rId22"/>
-    <sheet name="default_footnotes" sheetId="23" r:id="rId23"/>
+    <sheet name="ard_statistics" sheetId="10" r:id="rId10"/>
+    <sheet name="listing_types" sheetId="11" r:id="rId11"/>
+    <sheet name="populations" sheetId="12" r:id="rId12"/>
+    <sheet name="datasets" sheetId="13" r:id="rId13"/>
+    <sheet name="default_header" sheetId="14" r:id="rId14"/>
+    <sheet name="default_footer" sheetId="15" r:id="rId15"/>
+    <sheet name="default_cells" sheetId="16" r:id="rId16"/>
+    <sheet name="default_layout" sheetId="17" r:id="rId17"/>
+    <sheet name="default_columns" sheetId="18" r:id="rId18"/>
+    <sheet name="default_style" sheetId="19" r:id="rId19"/>
+    <sheet name="default_col_header" sheetId="20" r:id="rId20"/>
+    <sheet name="default_report" sheetId="21" r:id="rId21"/>
+    <sheet name="default_page" sheetId="22" r:id="rId22"/>
+    <sheet name="default_titles" sheetId="23" r:id="rId23"/>
+    <sheet name="default_footnotes" sheetId="24" r:id="rId24"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -373,7 +374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -520,78 +521,95 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>the ARD methods (keywords): the function, its kind (continuous / categorical / none, for statistic =), default arguments (&lt;id&gt; = the subject key) and statistics</t>
+          <t>the ARD methods (keywords): the function, its kind (continuous / categorical / missing / none, for statistic =), default arguments (&lt;id&gt; = the subject key), statistics and formats</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARD の手法キーワード：関数、種類（statistic の形）、既定の引数（&lt;id&gt; = 被験者キー）、統計量</t>
+          <t>ARD の手法キーワード：関数、種類（statistic の形）、既定の引数（&lt;id&gt; = 被験者キー）、統計量、書式</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>listing_types</t>
+          <t>ard_statistics</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>the listing types a listing may use (rtfreporter's)</t>
+          <t>the statistics an ARD analysis may ask for: kind, label, default format of stat_fmt (xx.x, xx.x%, pvalue), and the R function of those tflplanner computes</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Listing の種類（rtfreporter のもの）</t>
+          <t>ARD の統計量：種類、ラベル、stat_fmt の既定の書式（xx.x, xx.x%, pvalue）、tflplanner が計算するものの R 関数</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>populations</t>
+          <t>listing_types</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>the analysis sets a new study's ARD definition starts with</t>
+          <t>the listing types a listing may use (rtfreporter's)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>新規試験の ARD 定義が最初に持つ解析対象集団</t>
+          <t>Listing の種類（rtfreporter のもの）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>datasets</t>
+          <t>populations</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>the data catalog a new study starts with: ADaM and SDTM datasets and their files</t>
+          <t>the analysis sets a new study's ARD definition starts with</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>新規試験が最初に持つデータカタログ（ADaM / SDTM とファイル）</t>
+          <t>新規試験の ARD 定義が最初に持つ解析対象集団</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>the data catalog a new study starts with: ADaM and SDTM datasets and their files</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>新規試験が最初に持つデータカタログ（ADaM / SDTM とファイル）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>default_&lt;sheet&gt;</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>the study-default rows a new study starts with, one sheet per definition sheet (default_header, default_footer, default_cells ...); {STUDY_ID} becomes the study's id</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>新規試験の「試験共通の既定」の行。定義シートごとに 1 シート。{STUDY_ID} は試験 ID に置き換わる</t>
         </is>
@@ -604,21 +622,41 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>statistic</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fmt</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>fun</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -627,17 +665,1458 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>multiline</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>multiline</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter's listing type: / separator, gutters, a blank row per record</t>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>n (non-missing values)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>the missing are counted by the method `missing`</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>median</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>p25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Q1 (25th percentile)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>p75</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Q3 (75th percentile)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>cards</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SE of the mean</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>function(x) stats::sd(x) / sqrt(length(x))</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>function(x) stats::var(x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cv</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CV (%)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>function(x) stats::sd(x) / mean(x) * 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>range</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Range (max - min)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>function(x) max(x) - min(x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>iqr</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>IQR (Q3 - Q1)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>function(x) diff(stats::quantile(x, c(0.25, 0.75), type = 2, names = FALSE))</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>function(x) sum(x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>p5</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>percentiles</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5th percentile</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>function(x) stats::quantile(x, 0.05, type = 2, names = FALSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>p10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>percentiles</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10th percentile</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>function(x) stats::quantile(x, 0.10, type = 2, names = FALSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>p90</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>percentiles</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>90th percentile</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>function(x) stats::quantile(x, 0.90, type = 2, names = FALSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>percentiles</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>95th percentile</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>function(x) stats::quantile(x, 0.95, type = 2, names = FALSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mean_lcl</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>confidence limits</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Mean: lower 95% confidence limit (t)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>function(x) (mean(x) - stats::qt(0.975, length(x) - 1) * stats::sd(x) / sqrt(length(x)))</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mean_ucl</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>confidence limits</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mean: upper 95% confidence limit (t)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>function(x) (mean(x) + stats::qt(0.975, length(x) - 1) * stats::sd(x) / sqrt(length(x)))</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>geo_mean</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Geometric mean</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else exp(mean(log(x)))</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>geo_sd</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Geometric SD</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else exp(stats::sd(log(x)))</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>geo_cv</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Geometric CV (%)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else sqrt(exp(stats::sd(log(x))^2) - 1) * 100</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>geo_lcl</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Geometric mean: lower 95% confidence limit</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else exp(mean(log(x)) - stats::qt(0.975, length(x) - 1) * stats::sd(log(x)) / sqrt(length(x)))</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>geo_ucl</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Geometric mean: upper 95% confidence limit</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else exp(mean(log(x)) + stats::qt(0.975, length(x) - 1) * stats::sd(log(x)) / sqrt(length(x)))</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>log_mean</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mean of log values</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>xx.xxx</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else mean(log(x))</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>log_sd</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>log scale</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SD of log values</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>xx.xxx</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>function(x) if (any(x &lt;= 0)) NA_real_ else stats::sd(log(x))</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>computed on log(x); NA when a value is 0 or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>counts</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>n (subjects / records in the level)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>counts</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>N (the denominator)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>counts</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Percent (n / N)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>xx.x%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>n_cum</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>counts</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Cumulative n</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>p_cum</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>counts</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Cumulative percent</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>xx.x%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>N_obs</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Number of records</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>N_miss</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>N_nonmiss</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Non-missing</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>p_miss</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Percent missing</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>xx.x%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>p_nonmiss</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Percent non-missing</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>xx.x%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>conf.low</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Lower confidence limit</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>conf.high</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Upper confidence limit</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>std.error</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Standard error</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>xx.xxx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>estimate1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Estimate of group 1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>estimate2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Estimate of group 2</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>statistic</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Test statistic</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Degrees of freedom</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>xx.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>p.value</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>pvalue</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>conf.level</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>estimates</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Confidence level</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>xx.xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>n.risk</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Number at risk</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>xx</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>n.event</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>survival</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Number of events</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>xx</t>
         </is>
       </c>
     </row>
@@ -648,31 +2127,21 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>population_id</t>
+          <t>type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>where</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>derive</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -681,108 +2150,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SAF</t>
+          <t>multiline</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADSL</t>
+          <t>multiline</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SAFFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TRTA = TRT01A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Safety set</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>FAS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>FASFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Full analysis set</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PPS</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PPROTFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Per-protocol set</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ENR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ENRLFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Enrolled</t>
+          <t>rtfreporter's listing type: / separator, gutters, a blank row per record</t>
         </is>
       </c>
     </row>
@@ -793,23 +2171,23 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>population_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>where</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -826,306 +2204,108 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>SAF</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>ADSL</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>data/adam/adsl.rds</t>
+          <t>SAFFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TRTA = TRT01A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Safety set</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>FAS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>data/adam/adae.rds</t>
+          <t>FASFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Full analysis set</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADLB</t>
+          <t>PPS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>data/adam/adlb.rds</t>
+          <t>PPROTFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Per-protocol set</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADVS</t>
+          <t>ENR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>data/adam/advs.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ADEG</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>data/adam/adeg.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ADEX</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>data/adam/adex.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ADCM</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>data/adam/adcm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ADMH</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>data/adam/admh.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ADTTE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>data/adam/adtte.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ADRS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>data/adam/adrs.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>data/sdtm/dm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AE</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>data/sdtm/ae.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>data/sdtm/cm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>data/sdtm/mh.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>EX</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>data/sdtm/ex.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>data/sdtm/lb.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>VS</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>data/sdtm/vs.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>data/sdtm/ds.rds</t>
+          <t>ENRLFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Enrolled</t>
         </is>
       </c>
     </row>
@@ -1136,28 +2316,28 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>level</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>path</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>derive</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1169,34 +2349,306 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data/adam/adsl.rds</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>ADAE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Protocol: {STUDY_ID}</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Page {PAGE} of {TOTAL_PAGES}</t>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>data/adam/adae.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADLB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>data/adam/adlb.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ADVS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>data/adam/advs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ADEG</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>data/adam/adeg.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ADEX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>data/adam/adex.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ADCM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>data/adam/adcm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ADMH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>data/adam/admh.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADTTE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>data/adam/adtte.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ADRS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>data/adam/adrs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>data/sdtm/dm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>data/sdtm/ae.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>data/sdtm/cm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>data/sdtm/mh.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>data/sdtm/ex.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>data/sdtm/lb.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>data/sdtm/vs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>data/sdtm/ds.rds</t>
         </is>
       </c>
     </row>
@@ -1207,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1240,12 +2692,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{PROGRAM}       Generated on: {DATETIME}</t>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Protocol: {STUDY_ID}</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Page {PAGE} of {TOTAL_PAGES}</t>
         </is>
       </c>
     </row>
@@ -1256,60 +2730,45 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>line</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>left</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>row</t>
+          <t>center</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>when</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>digits</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>signif</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>{n:.0f} ({p:.1f%})</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>every categorical cell</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{PROGRAM}       Generated on: {DATETIME}</t>
         </is>
       </c>
     </row>
@@ -1320,160 +2779,60 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>pages_max_rows</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>pages_split</t>
+          <t>context</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pages_by</t>
+          <t>row</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>pages_min_group_rows</t>
+          <t>when</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pages_cont_label</t>
+          <t>template</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>group_col</t>
+          <t>digits</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>group_mode</t>
+          <t>signif</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>group_collapse</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>group_page</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>group_show</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>blank_where</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>blank_first</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>blank_last</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>blank_counted</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>stub_vars</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>stub_into</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>stub_indent</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>stub_summary</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>stub_before</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_every</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_at</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_carry</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_order</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>between_groups</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>row_label</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{n:.0f} ({p:.1f%})</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>every categorical cell</t>
         </is>
       </c>
     </row>
@@ -1484,62 +2843,160 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>column</t>
+          <t>pages_max_rows</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>width</t>
+          <t>pages_split</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>row_title</t>
+          <t>pages_by</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>decimal_split</t>
+          <t>pages_min_group_rows</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>hide</t>
+          <t>pages_cont_label</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>group_col</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>group_mode</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>group_collapse</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>group_page</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>group_show</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>blank_where</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>blank_first</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>blank_last</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>blank_counted</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>stub_vars</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>stub_into</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>stub_indent</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>stub_summary</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>stub_before</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_every</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_at</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_carry</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_order</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>between_groups</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>row_label</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>.values</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>18</t>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1550,70 +3007,62 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>border</t>
+          <t>column</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>align_count_pct</t>
+          <t>width</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>auto_width</t>
+          <t>row_title</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>row_height_twips</t>
+          <t>decimal_split</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>header_row_height_twips</t>
+          <t>hide</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>blank_row_height_twips</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>font</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>font_size_half_points</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>table_align</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>cell_valign</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -1624,126 +3073,70 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>border</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>cols</t>
+          <t>align_count_pct</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>span</t>
+          <t>auto_width</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>row_height_twips</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>align</t>
+          <t>header_row_height_twips</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>bold</t>
+          <t>blank_row_height_twips</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>border_top</t>
+          <t>font</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>border_bottom</t>
+          <t>font_size_half_points</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>table_align</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>cell_valign</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>row_label</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>.values</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>{col}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>row_label</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>.values</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>(N={n})</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1819,71 +3212,51 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>line</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>cols</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>span</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>auto_section</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>section_align</t>
+          <t>align</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>auto_title</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>title_align</t>
+          <t>border_top</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>table_font_size</t>
+          <t>border_bottom</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>title_font_size</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>footnote_font_size</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>page_header</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>page_footer</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1892,17 +3265,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{output_id}.rtf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>{output_id}.R</t>
+          <t>row_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{col}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Characteristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(N={n})</t>
         </is>
       </c>
     </row>
@@ -1913,93 +3342,90 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>paper_size</t>
+          <t>type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>orientation</t>
+          <t>file</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>width_in</t>
+          <t>program</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>height_in</t>
+          <t>auto_section</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>margin_top_in</t>
+          <t>section_align</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>margin_bottom_in</t>
+          <t>auto_title</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>margin_left_in</t>
+          <t>title_align</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>margin_right_in</t>
+          <t>table_font_size</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>header_dist_in</t>
+          <t>title_font_size</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>footer_dist_in</t>
+          <t>footnote_font_size</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>font_size_half_points</t>
+          <t>page_header</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>title_format</t>
+          <t>page_footer</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>footnote_format</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>title_width</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>footnote_width</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>markup</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{output_id}.rtf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>{output_id}.R</t>
         </is>
       </c>
     </row>
@@ -2010,31 +3436,91 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>paper_size</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>orientation</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>width_in</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>height_in</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>margin_top_in</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>margin_bottom_in</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>margin_left_in</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>margin_right_in</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>header_dist_in</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>footer_dist_in</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>font_size_half_points</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>title_format</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_format</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>title_width</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_width</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>markup</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2082,6 +3568,43 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C7"/>
@@ -4306,7 +5829,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4337,6 +5860,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>formats</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -4357,7 +5885,7 @@
           <t>continuous</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>summary statistics of numeric variables</t>
         </is>
@@ -4379,7 +5907,7 @@
           <t>categorical</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>counts and percents of each level</t>
         </is>
@@ -4401,7 +5929,7 @@
           <t>categorical</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>counts of one level (args: value = list(VAR = "Y"))</t>
         </is>
@@ -4420,10 +5948,10 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>missing and non-missing counts</t>
         </is>
@@ -4450,7 +5978,7 @@
           <t>denominator = population, id = &lt;id&gt;</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>nested subject counts, outermost variable first (SOC | PT)</t>
         </is>
@@ -4464,7 +5992,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cardx::ard_categorical_max</t>
+          <t>cardx::ard_tabulate_max</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4477,7 +6005,7 @@
           <t>denominator = population, id = &lt;id&gt;</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>the worst level per subject; variables = the graded variable</t>
         </is>
@@ -4499,7 +6027,7 @@
           <t>categorical</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>subjects with a record of the data (after where); variables = a name for the count</t>
         </is>
@@ -4521,7 +6049,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>number of subjects</t>
         </is>
@@ -4545,7 +6073,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>confidence interval of a proportion (args: method = "wilson" ...)</t>
+          <t>estimate=xx.x% | conf.low=xx.x% | conf.high=xx.x%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>confidence interval of a proportion (args: method = "wilson" ...); statistics keep some of estimate, conf.low, conf.high</t>
         </is>
       </c>
     </row>
@@ -4567,27 +6100,120 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>confidence interval of a mean</t>
+          <t>estimate=xx.x | conf.low=xx.x | conf.high=xx.x</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>confidence interval of a mean (args: conf.level = 0.9 ...); statistics keep some of estimate, conf.low, conf.high</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ttest</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cardx::ard_stats_t_test</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>two-sample t test between the `by` groups (two of them)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>wilcox</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cardx::ard_stats_wilcox_test</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Wilcoxon rank-sum test between the `by` groups (two of them)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>chisq</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cardx::ard_stats_chisq_test</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>chi-square test of variables x by</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fisher</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cardx::ard_stats_fisher_test</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Fisher's exact test of variables x by</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>(code)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>any R code in `code`; data and population are bound</t>
         </is>

</xml_diff>

<commit_message>
ARD programs one per output (programs/ard/), autoexec_ard.R, and run logs
- programs/ard/: ard_setup.R (sourced), <output_id>.R per output (replaces
  its rows of the study ARD, records the build), autoexec_ard.R
- programs/tfl/: the report programs and autoexec_report.R (no longer runs
  the ARD); earlier studies' programs move there on save
- every program runs in its own R process via R CMD BATCH (code and output,
  plus who/where/which R) or logrx::axecute() (standards: log_engine);
  logs in logs/ard/ and logs/tfl/
- the app builds the study ARD from the saved programs only; Study ARD shows
  each output's log; the Code panel shows the program / ard_setup.R /
  autoexec_ard.R with its state on disk

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/standards/company_standards_draft.xlsx
+++ b/inst/standards/company_standards_draft.xlsx
@@ -3607,7 +3607,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3721,6 +3721,23 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>a key with more levels gets no levels list when filled from the ARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>log_engine</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>how programs are run and logged: batch (R CMD BATCH: the code and its output) or logrx (logrx::axecute(), when installed)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Follow tflspec's column names and help; fingerprints read `source`
tflspec renamed columns$width to rel_width and the report's
table/title/footnote_font_size to *_font_size_half_points
(ichirio/tflspec#64): the company standards' default columns, their draft
workbook and the sample study SAMPLE-01 (made again; its eight reports'
RTFs are byte-identical to before but for the run time) follow.

tflspec's column help is English now: the help tables show it through
tr(), with the Japanese of every description in strings.csv.

tfl_ard_spec_hash() reads the study's own function files (key `source`):
ard_program_code() gains `dir`, and the programs, the Code view and
ard_status() pass the study folder.  Needs tflspec 0.0.24.9011.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/standards/company_standards_draft.xlsx
+++ b/inst/standards/company_standards_draft.xlsx
@@ -17,20 +17,24 @@
     <sheet name="categorical_formats" sheetId="8" r:id="rId8"/>
     <sheet name="ard_methods" sheetId="9" r:id="rId9"/>
     <sheet name="ard_statistics" sheetId="10" r:id="rId10"/>
-    <sheet name="listing_types" sheetId="11" r:id="rId11"/>
-    <sheet name="populations" sheetId="12" r:id="rId12"/>
-    <sheet name="datasets" sheetId="13" r:id="rId13"/>
-    <sheet name="default_header" sheetId="14" r:id="rId14"/>
-    <sheet name="default_footer" sheetId="15" r:id="rId15"/>
-    <sheet name="default_cells" sheetId="16" r:id="rId16"/>
-    <sheet name="default_layout" sheetId="17" r:id="rId17"/>
-    <sheet name="default_columns" sheetId="18" r:id="rId18"/>
-    <sheet name="default_style" sheetId="19" r:id="rId19"/>
-    <sheet name="default_col_header" sheetId="20" r:id="rId20"/>
-    <sheet name="default_report" sheetId="21" r:id="rId21"/>
-    <sheet name="default_page" sheetId="22" r:id="rId22"/>
-    <sheet name="default_titles" sheetId="23" r:id="rId23"/>
-    <sheet name="default_footnotes" sheetId="24" r:id="rId24"/>
+    <sheet name="figure_settings" sheetId="11" r:id="rId11"/>
+    <sheet name="figure_colors" sheetId="12" r:id="rId12"/>
+    <sheet name="figure_markers" sheetId="13" r:id="rId13"/>
+    <sheet name="code_templates" sheetId="14" r:id="rId14"/>
+    <sheet name="listing_types" sheetId="15" r:id="rId15"/>
+    <sheet name="populations" sheetId="16" r:id="rId16"/>
+    <sheet name="datasets" sheetId="17" r:id="rId17"/>
+    <sheet name="default_header" sheetId="18" r:id="rId18"/>
+    <sheet name="default_footer" sheetId="19" r:id="rId19"/>
+    <sheet name="default_cells" sheetId="20" r:id="rId20"/>
+    <sheet name="default_layout" sheetId="21" r:id="rId21"/>
+    <sheet name="default_columns" sheetId="22" r:id="rId22"/>
+    <sheet name="default_style" sheetId="23" r:id="rId23"/>
+    <sheet name="default_col_header" sheetId="24" r:id="rId24"/>
+    <sheet name="default_report" sheetId="25" r:id="rId25"/>
+    <sheet name="default_page" sheetId="26" r:id="rId26"/>
+    <sheet name="default_titles" sheetId="27" r:id="rId27"/>
+    <sheet name="default_footnotes" sheetId="28" r:id="rId28"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -374,7 +378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -550,66 +554,134 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>listing_types</t>
+          <t>figure_settings</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>the listing types a listing may use (rtfreporter's)</t>
+          <t>the figure style: one value per key (type blank = every figure; km / waterfall / swimmer = that type)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Listing の種類（rtfreporter のもの）</t>
+          <t>図のスタイル：キーごとに 1 つの値（type 空欄 = すべての図、km / waterfall / swimmer = その種類だけ）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>populations</t>
+          <t>figure_colors</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>the analysis sets a new study's ARD definition starts with</t>
+          <t>the figure palettes: a named palette colours the values it names (response: CR, PR ...); one with value blank is used in order (treatment)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>新規試験の ARD 定義が最初に持つ解析対象集団</t>
+          <t>図のパレット：値の名前付き（response：CR、PR など）はその値の色、value 空欄（treatment）は順番に使う</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>datasets</t>
+          <t>figure_markers</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>the data catalog a new study starts with: ADaM and SDTM datasets and their files</t>
+          <t>the figure markers: event markers by label (Death, Discontinued ...) and the figures' symbols (censor, assessment)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>新規試験が最初に持つデータカタログ（ADaM / SDTM とファイル）</t>
+          <t>図の記号：ラベルごとのイベント記号（Death、Discontinued など）と図の記号（censor、assessment）</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>code_templates</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>the code written where a report says none: table_data (its rows of the study ARD), table_process (normalize, rework), figure_plot, setup; {OUTPUT_ID} {ARD} {ARD_PROGRAM} {PROGRAM} {STUDY_ID} are filled in</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>帳票が何も書かないときのコード：table_data（ARD からの取得）、table_process（normalize・加工）、figure_plot、setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>listing_types</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>the listing types a listing may use (rtfreporter's)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Listing の種類（rtfreporter のもの）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>populations</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>the analysis sets a new study's ARD definition starts with</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>新規試験の ARD 定義が最初に持つ解析対象集団</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>the data catalog a new study starts with: ADaM and SDTM datasets and their files</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>新規試験が最初に持つデータカタログ（ADaM / SDTM とファイル）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>default_&lt;sheet&gt;</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>the study-default rows a new study starts with, one sheet per definition sheet (default_header, default_footer, default_cells ...); {STUDY_ID} becomes the study's id</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>新規試験の「試験共通の既定」の行。定義シートごとに 1 シート。{STUDY_ID} は試験 ID に置き換わる</t>
         </is>
@@ -2127,7 +2199,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2138,29 +2210,1051 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>key</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>multiline</t>
+          <t>base_size</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter's listing type: / separator, gutters, a blank row per record</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>base font size (pt) of the theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>axis_title_size</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>axis titles (pt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>axis_text_size</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>axis tick labels (pt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>legend_text_size</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>legend text (pt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>legend_key_size</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>legend key size (lines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>text_size</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>text drawn in the panel (mm, geom_text size)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>theme</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>boxed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>boxed | L_axis | minimal | classic</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>panel_border_width</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>boxed: panel border (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>axis_line_width</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>L_axis: axis lines (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tick_width</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>axis ticks (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tick_length</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>axis tick length (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>line_width</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>data lines (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>zero_line_colour</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>reference line at 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>zero_line_width</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ref_line_colour</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>grey</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>threshold lines (e.g. +20% / -30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ref_linetype</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>dashed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ref_line_width</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>month_days</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30.4375</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>days in a month, for day -&gt; month axes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>output size</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>in | cm | px</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>dpi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>censor_shape</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>censor mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>censor_size</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>censor_stroke</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>median_linetype</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>twodash</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>the 50% line</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>median_colour</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>grey50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>median_line_width</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>y_by</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>survival axis breaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>risk_title</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Number of Patients at Risk</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>number at risk panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>risk_height</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0.167</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>number at risk panel / curve height (1:6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>8.33</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2500 x 1438 px at 300 dpi</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>4.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>bar_width</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ref_lines</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>20,-30</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>threshold lines (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ref_label_size</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>labels of the threshold lines (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ref_label_hjust</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>-0.3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>outside the panel, right</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>right_margin</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>room for the labels (pt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>y_min</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>-100</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>y_max</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>y_by</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>waterfall</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>x_label</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>theme</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>L_axis</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>bar_width</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>subject bars (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>marker_size</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>marker_palette</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>event_size</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>event markers</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>visit_linetype</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>dotted</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>visit grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>visit_colour</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>visit_label</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>bar_legend_prefix</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Best response</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>legend label: &lt;prefix&gt; &lt;response&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>legend_ncol</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>legend panel below the plot</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>legend_height</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>legend panel / plot height (1:5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>legend_point_size</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>legend_label_size</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>(mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>7.71</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>swimmer</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>4.17</t>
         </is>
       </c>
     </row>
@@ -2171,31 +3265,26 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>population_id</t>
+          <t>palette</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>where</t>
+          <t>colour</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>derive</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2204,108 +3293,575 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SAF</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ADSL</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SAFFL == "Y"</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TRTA = TRT01A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Safety set</t>
+          <t>KM sample (single arm)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FAS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FASFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Full analysis set</t>
+          <t>#D55E00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PPS</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ADSL</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PPROTFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Per-protocol set</t>
+          <t>#009E73</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ENR</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ADSL</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ENRLFL == "Y"</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TRTP = TRT01P</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Enrolled</t>
+          <t>#CC79A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>treatment</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#E69F00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>treatment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#56B4E9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>waterfall sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#0000FF</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>waterfall sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#FFA500</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>waterfall sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>#800080</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>waterfall sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>#A0A0A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NON-CR/NON-PD</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>#20B2AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>swimmer sample: the response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>#0000CD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>swimmer sample: the response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>#FF8C00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>swimmer sample: the response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>#9400D3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>swimmer sample: the response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>response_assessment</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>swimmer sample: the response at each assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>#99CC99</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>swimmer sample: best overall response</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>#9999FF</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>swimmer sample: best overall response</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>#FFCC99</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>swimmer sample: best overall response</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>#CC99FF</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>swimmer sample: best overall response</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>#D9D9D9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>response_light</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>NON-CR/NON-PD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>#99D8D3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>#E69F00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>#56B4E9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>#009E73</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>#F0E442</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>#0072B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>#D55E00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>#CC79A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>okabe_ito</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>#000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>grey</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>#000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>grey</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>#555555</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>grey</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>#999999</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>grey</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>#CCCCCC</t>
         </is>
       </c>
     </row>
@@ -2316,31 +3872,36 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>shape</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>fill</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>derive</t>
+          <t>colour</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2349,306 +3910,167 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADSL</t>
+          <t>Death</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>data/adam/adsl.rds</t>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>transparent</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>swimmer sample</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>Subsequent anti-cancer therapy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>data/adam/adae.rds</t>
+          <t>#FF00FF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>transparent</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>swimmer sample</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADLB</t>
+          <t>Discontinued</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADaM</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>data/adam/adlb.rds</t>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>transparent</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>swimmer sample</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADVS</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>data/adam/advs.rds</t>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>transparent</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>swimmer sample: response at each assessment (fill = response)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADEG</t>
+          <t>best_response</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>data/adam/adeg.rds</t>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>legend of the best-response bars</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADEX</t>
+          <t>censor</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>data/adam/adex.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ADCM</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>data/adam/adcm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ADMH</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>data/adam/admh.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ADTTE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>data/adam/adtte.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ADRS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ADaM</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>data/adam/adrs.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>data/sdtm/dm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AE</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>data/sdtm/ae.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>data/sdtm/cm.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>data/sdtm/mh.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>EX</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>data/sdtm/ex.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>data/sdtm/lb.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>VS</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>data/sdtm/vs.rds</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DS</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SDTM</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>data/sdtm/ds.rds</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>KM sample: x</t>
         </is>
       </c>
     </row>
@@ -2659,31 +4081,21 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2692,34 +4104,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>table_data</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
+          <t># ---- this output's rows of the study ARD ({ARD}, made by {ARD_PROGRAM})
+ard &lt;- readRDS("{ARD}")
+ard &lt;- ard[ard$output_id == "{OUTPUT_ID}",
+           setdiff(names(ard), c("output_id", "analysis_id", "population_id"))]
+if (!nrow(ard)) stop("The study ARD has no rows for {OUTPUT_ID}: make its ARD first.")</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a table's data code when it has none: its rows of the study ARD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>table_process</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Protocol: {STUDY_ID}</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Page {PAGE} of {TOTAL_PAGES}</t>
+          <t># ---- normalize
+data &lt;- normalize_ard(ard)
+# ---- rework as needed, e.g.
+# data &lt;- dplyr::mutate(data, label = dplyr::recode(label, "Age" = "Age (years)"))</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>a table's normalization when it has none: after table_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>figure_plot</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t># TODO: the plot (ggplot2), in the figure style of the company standards, e.g.
+#   plot &lt;- ggplot2::ggplot(adsl, ggplot2::aes(AGE, fill = TRT01A)) +
+#     ggplot2::geom_histogram() + scale_fill_tfl("treatment", levels(adsl$TRT01A)) +
+#     theme_tfl()</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>a figure's plot before it is written (a stop() follows it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>setup</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>the setup code every report of a new study runs first (blank: none)</t>
         </is>
       </c>
     </row>
@@ -2730,31 +4181,21 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2763,12 +4204,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>multiline</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{PROGRAM}       Generated on: {DATETIME}</t>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>rtfreporter's listing type: / separator, gutters, a blank row per record</t>
         </is>
       </c>
     </row>
@@ -2779,60 +4225,141 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>population_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>row</t>
+          <t>where</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>when</t>
+          <t>derive</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>digits</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>signif</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SAF</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SAFFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TRTA = TRT01A</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{n:.0f} ({p:.1f%})</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>every categorical cell</t>
+          <t>Safety set</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FAS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FASFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Full analysis set</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PPS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PPROTFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Per-protocol set</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ENR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ENRLFL == "Y"</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TRTP = TRT01P</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Enrolled</t>
         </is>
       </c>
     </row>
@@ -2843,160 +4370,339 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>pages_max_rows</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>pages_split</t>
+          <t>level</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pages_by</t>
+          <t>path</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>pages_min_group_rows</t>
+          <t>derive</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pages_cont_label</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>group_col</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>group_mode</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>group_collapse</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>group_page</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>group_show</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>blank_where</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>blank_first</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>blank_last</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>blank_counted</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>stub_vars</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>stub_into</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>stub_indent</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>stub_summary</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>stub_before</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_every</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_at</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_carry</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_order</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>between_groups</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>row_label</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>data/adam/adsl.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADAE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>data/adam/adae.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADLB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>data/adam/adlb.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ADVS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>data/adam/advs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ADEG</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>data/adam/adeg.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ADEX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>data/adam/adex.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ADCM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>data/adam/adcm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ADMH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>data/adam/admh.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADTTE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>data/adam/adtte.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ADRS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>data/adam/adrs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>data/sdtm/dm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>data/sdtm/ae.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>data/sdtm/cm.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>data/sdtm/mh.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>data/sdtm/ex.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>data/sdtm/lb.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>data/sdtm/vs.rds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SDTM</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>data/sdtm/ds.rds</t>
         </is>
       </c>
     </row>
@@ -3007,36 +4713,31 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>column</t>
+          <t>line</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>width</t>
+          <t>left</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>row_title</t>
+          <t>center</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>decimal_split</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>hide</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -3045,24 +4746,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>row_label</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>.values</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>Protocol: {STUDY_ID}</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Page {PAGE} of {TOTAL_PAGES}</t>
         </is>
       </c>
     </row>
@@ -3073,70 +4784,45 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>border</t>
+          <t>line</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>align_count_pct</t>
+          <t>left</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>auto_width</t>
+          <t>center</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>row_height_twips</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>header_row_height_twips</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>blank_row_height_twips</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>font</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>font_size_half_points</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>table_align</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>cell_valign</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>{PROGRAM}       Generated on: {DATETIME}</t>
         </is>
       </c>
     </row>
@@ -3212,126 +4898,60 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>cols</t>
+          <t>context</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>span</t>
+          <t>row</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>when</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>align</t>
+          <t>template</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>bold</t>
+          <t>digits</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>border_top</t>
+          <t>signif</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>border_bottom</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>row_label</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>.values</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>{col}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>row_label</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>.values</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>(N={n})</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{n:.0f} ({p:.1f%})</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>every categorical cell</t>
         </is>
       </c>
     </row>
@@ -3342,90 +4962,175 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>pages_max_rows</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>pages_split</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>pages_break_before</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>auto_section</t>
+          <t>pages_min_group_rows</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>section_align</t>
+          <t>pages_cont_label</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>auto_title</t>
+          <t>group_col</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>title_align</t>
+          <t>group_mode</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>table_font_size</t>
+          <t>group_collapse</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>title_font_size</t>
+          <t>group_page</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>footnote_font_size</t>
+          <t>group_keep</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>page_header</t>
+          <t>blank_where</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>page_footer</t>
+          <t>blank_first</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>blank_last</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>blank_counted</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>stub_vars</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>stub_name</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>stub_indent</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>stub_summary</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>stub_before</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_every</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_at</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_keep</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_order</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_cut_by</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_fit</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>colpages_allow_span_break</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>table</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>{output_id}.rtf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>{output_id}.R</t>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>between_groups</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3436,93 +5141,62 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>paper_size</t>
+          <t>column</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>orientation</t>
+          <t>rel_width</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>width_in</t>
+          <t>row_title</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>height_in</t>
+          <t>decimal_split</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>margin_top_in</t>
+          <t>hide</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>margin_bottom_in</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>margin_left_in</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>margin_right_in</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>header_dist_in</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>footer_dist_in</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>font_size_half_points</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>title_format</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>footnote_format</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>title_width</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>footnote_width</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>markup</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
           <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -3533,33 +5207,120 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>border</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>align_count_pct</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>auto_width</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>row_height_twips</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>row_height_exact</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>header_row_height_twips</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>blank_row_height_twips</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>cell_padding_left_twips</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>cell_padding_right_twips</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>font</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>font_size_half_points</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>table_align</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>cell_valign</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>markup</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>blank_row_normalize</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>border_header</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>border_spanning</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>border_body</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>border_first_row</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>border_last_row</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -3569,6 +5330,364 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cols</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>span</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>align</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>bold</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>border_top</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>border_bottom</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{col}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>row_label</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Characteristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>.values</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(N={n})</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>auto_section</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>section_align</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>auto_title</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>title_align</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>table_font_size_half_points</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>title_font_size_half_points</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_font_size_half_points</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>page_header</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>page_footer</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{output_id}.rtf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>{output_id}.R</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>paper_size</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>orientation</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>height_in</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>margin_top_in</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>margin_bottom_in</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>margin_left_in</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>margin_right_in</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>header_dist_in</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>footer_dist_in</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>font_size_half_points</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>title_format</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_format</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>title_width</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>footnote_width</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>markup</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3710,34 +5829,29 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>max_levels</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>30</t>
+          <t>listing_max_rows</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>a key with more levels gets no levels list when filled from the ARD</t>
+          <t>the rows per page a new listing starts with (blank: as many as fit, rtfreporter's)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>log_engine</t>
+          <t>max_levels</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>batch</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>how programs are run and logged: batch (R CMD BATCH: the code and its output) or logrx (logrx::axecute(), when installed)</t>
+          <t>a key with more levels gets no levels list when filled from the ARD</t>
         </is>
       </c>
     </row>
@@ -3963,7 +6077,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>group_show</t>
+          <t>group_keep</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3980,7 +6094,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>group_show</t>
+          <t>group_keep</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5846,7 +7960,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -5857,30 +7971,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>call</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>statistics</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>formats</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -5894,15 +8013,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Summary statistics</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>cards::ard_continuous</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>continuous</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>summary statistics of numeric variables</t>
         </is>
@@ -5916,15 +8040,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Counts and percents</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>cards::ard_categorical</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>counts and percents of each level</t>
         </is>
@@ -5938,15 +8067,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Count of one level</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>cards::ard_dichotomous</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>counts of one level (args: value = list(VAR = "Y"))</t>
         </is>
@@ -5960,15 +8094,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Missing counts</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>cards::ard_missing</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>missing and non-missing counts</t>
         </is>
@@ -5982,20 +8121,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Nested counts (e.g. SOC / PT)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>cards::ard_stack_hierarchical</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>denominator = population, id = &lt;id&gt;</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>nested subject counts, outermost variable first (SOC | PT)</t>
         </is>
@@ -6009,20 +8153,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Worst level per subject</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>cardx::ard_tabulate_max</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>denominator = population, id = &lt;id&gt;</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>the worst level per subject; variables = the graded variable</t>
         </is>
@@ -6036,15 +8185,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Subjects with a record</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>(subjects)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>categorical</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>subjects with a record of the data (after where); variables = a name for the count</t>
         </is>
@@ -6058,15 +8212,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Number of subjects</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>cards::ard_total_n</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>number of subjects</t>
         </is>
@@ -6080,20 +8239,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Proportion with CI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>cardx::ard_categorical_ci</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>estimate=xx.x% | conf.low=xx.x% | conf.high=xx.x%</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>confidence interval of a proportion (args: method = "wilson" ...); statistics keep some of estimate, conf.low, conf.high</t>
         </is>
@@ -6107,20 +8271,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Mean with CI</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>cardx::ard_continuous_ci</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>estimate=xx.x | conf.low=xx.x | conf.high=xx.x</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>confidence interval of a mean (args: conf.level = 0.9 ...); statistics keep some of estimate, conf.low, conf.high</t>
         </is>
@@ -6134,15 +8303,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>t test</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>cardx::ard_stats_t_test</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>two-sample t test between the `by` groups (two of them)</t>
         </is>
@@ -6156,15 +8330,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Wilcoxon rank-sum test</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>cardx::ard_stats_wilcox_test</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Wilcoxon rank-sum test between the `by` groups (two of them)</t>
         </is>
@@ -6178,15 +8357,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Chi-square test</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>cardx::ard_stats_chisq_test</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>chi-square test of variables x by</t>
         </is>
@@ -6200,15 +8384,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Fisher's exact test</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>cardx::ard_stats_fisher_test</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Fisher's exact test of variables x by</t>
         </is>
@@ -6222,15 +8411,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Custom R code</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>(code)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>any R code in `code`; data and population are bound</t>
         </is>

</xml_diff>